<commit_message>
M4 entero con el vuelo lateral (3,80 m) y regla de precio cerrado con NIDO
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/costes/Nevola_piloto_estudio_costes.xlsx
+++ b/costes/Nevola_piloto_estudio_costes.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="342">
   <si>
     <t>NÉVOLA · VIVIENDA PILOTO EN SISTEMA MODULAR · ESTUDIO DE COSTES</t>
   </si>
@@ -44,7 +44,7 @@
     <t>Sobrecoste de primera unidad en mano de obra de fábrica</t>
   </si>
   <si>
-    <t>Transporte de 6 módulos + pieza de vuelo</t>
+    <t>Transporte de 6 módulos, con el M4 como especial</t>
   </si>
   <si>
     <t>Grúa (jornada completa)</t>
@@ -62,10 +62,10 @@
     <t>COSTE DEL PILOTO</t>
   </si>
   <si>
-    <t>Margen RG21</t>
-  </si>
-  <si>
-    <t>PRECIO DEL PILOTO (sin IVA)</t>
+    <t>Margen RG21 (precio cerrado menos coste)</t>
+  </si>
+  <si>
+    <t>PRECIO CERRADO CON NIDO (sin IVA)</t>
   </si>
   <si>
     <t>€/m² construido</t>
@@ -206,10 +206,10 @@
     <t>Sotopinilla 2024: 780 €</t>
   </si>
   <si>
-    <t>Transporte de la pieza de vuelo lateral (0,60 × 8,47 m)</t>
-  </si>
-  <si>
-    <t>Estimado: viaje aparte en camión pluma</t>
+    <t>Suplemento de transporte especial del M4 (3,80 m de ancho, con acompañamiento)</t>
+  </si>
+  <si>
+    <t>ESTIMADO: pedir precio al transportista</t>
   </si>
   <si>
     <t>Grúa: jornada completa (coste 2024 €)</t>
@@ -248,7 +248,10 @@
     <t>Primera unidad sin otras obras en la nave</t>
   </si>
   <si>
-    <t>Margen RG21 (GG + beneficio)</t>
+    <t>Margen de referencia con el que se calculó la oferta (el precio ya está cerrado)</t>
+  </si>
+  <si>
+    <t>Oferta aceptada por NIDO: 225.400 € piloto, 209.100 € pareada en serie</t>
   </si>
   <si>
     <t>GG + BI de una contrata tradicional sobre PEM</t>
@@ -257,7 +260,7 @@
     <t>MODULACIÓN DE LA VIVIENDA PAREADA (piloto)</t>
   </si>
   <si>
-    <t>Seis módulos de acero, tres por planta, sin cambiar la distribución: anchos de 3,20 / 2,30 / 2,35 m (juntas a 3,20 y 5,50 m en planta baja). La planta primera vuela 0,60 m en frente y lateral; el vuelo lateral es una pieza aparte (V) que se atornilla al M4 en parcela. La junta a 3,20 m cruza el dormitorio 1 y se oculta en suelo y techo.</t>
+    <t>Seis módulos de acero, tres por planta, sin cambiar la distribución: anchos de 3,20 / 2,30 / 2,35 m (juntas a 3,20 y 5,50 m en planta baja). La planta primera vuela 0,60 m en frente y lateral; el vuelo lateral va dentro del M4, que mide 3,80 m de ancho. La junta a 3,20 m cruza el dormitorio 1 y se oculta en suelo y techo.</t>
   </si>
   <si>
     <t>Módulo</t>
@@ -308,7 +311,7 @@
     <t>P1</t>
   </si>
   <si>
-    <t>Dormitorio 3, baño 2, dormitorio principal · vuelo frontal 0,60</t>
+    <t>Dormitorio 3, baño 2, dormitorio principal · vuelos frontal y lateral de 0,60 dentro del módulo</t>
   </si>
   <si>
     <t>M5</t>
@@ -323,16 +326,10 @@
     <t>Dormitorio 2, escalera, vestidor, baño principal (medianera)</t>
   </si>
   <si>
-    <t>V</t>
-  </si>
-  <si>
-    <t>Pieza de vuelo lateral, se monta en parcela (no es módulo volumétrico)</t>
-  </si>
-  <si>
     <t>TOTAL</t>
   </si>
   <si>
-    <t>Transporte: el módulo más alto mide unos 3,05 m; en góndola rebajada (0,85 m) queda en ≈ 3,90 m, dentro del límite de 4,00 m. Ningún módulo pasa de 3,20 m de ancho: todos viajan sin transporte especial. La pieza de vuelo va aparte.</t>
+    <t>Transporte: el módulo más alto mide unos 3,05 m; en góndola rebajada (0,85 m) queda en ≈ 3,90 m, dentro del límite de 4,00 m. Todos superan 2,55 m de ancho y viajan con autorización especial; el M4, de 3,80 m, además con vehículo de acompañamiento.</t>
   </si>
   <si>
     <t>MEDICIÓN DE ACERO POR ELEMENTO (tipología del proyecto de Mahón 182)</t>
@@ -371,16 +368,10 @@
     <t>Viga de borde frontal en vuelo IPE 220</t>
   </si>
   <si>
+    <t>Viga de borde lateral en vuelo IPE 220</t>
+  </si>
+  <si>
     <t>Pilares IPE 160 (8 ud × 2.65 m)</t>
-  </si>
-  <si>
-    <t>Vuelo</t>
-  </si>
-  <si>
-    <t>Voladizo lateral 0,60 × 8,47: bordes IPE 220</t>
-  </si>
-  <si>
-    <t>Voladizo lateral: ménsulas IPE 160 cada 1,5 m (7 ud × 2 × 0,60)</t>
   </si>
   <si>
     <t>General</t>
@@ -1595,10 +1586,10 @@
         <v>7</v>
       </c>
       <c r="B7" s="5">
-        <f>(Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.59*Supuestos!$B$8*Supuestos!$B$7)*Supuestos!$B$21</f>
+        <f>(Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.61*Supuestos!$B$8*Supuestos!$B$7)*Supuestos!$B$21</f>
       </c>
       <c r="C7" s="5">
-        <f>(Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.59*Supuestos!$B$8*Supuestos!$B$7)*Supuestos!$B$21</f>
+        <f>(Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.61*Supuestos!$B$8*Supuestos!$B$7)*Supuestos!$B$21</f>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1672,10 +1663,10 @@
         <v>14</v>
       </c>
       <c r="B14" s="5">
-        <f>B13*Supuestos!$B$31</f>
+        <f>B15-B13</f>
       </c>
       <c r="C14" s="5">
-        <f>C13*Supuestos!$B$31</f>
+        <f>C15-C13</f>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -1683,10 +1674,10 @@
         <v>15</v>
       </c>
       <c r="B15" s="7">
-        <f>B13+B14</f>
+        <f>225400</f>
       </c>
       <c r="C15" s="7">
-        <f>C13+C14</f>
+        <f>273600</f>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -2028,7 +2019,7 @@
         <v>62</v>
       </c>
       <c r="B23" s="13">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>63</v>
@@ -2119,12 +2110,12 @@
         <v>0.1</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>17</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B32" s="10">
         <v>0.19</v>
@@ -2159,43 +2150,43 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C5" s="15">
         <v>3.2</v>
@@ -2210,15 +2201,15 @@
         <f>C5*D5</f>
       </c>
       <c r="G5" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C6" s="15">
         <v>2.3</v>
@@ -2233,15 +2224,15 @@
         <f>C6*D6</f>
       </c>
       <c r="G6" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C7" s="15">
         <v>2.35</v>
@@ -2256,18 +2247,18 @@
         <f>C7*D7</f>
       </c>
       <c r="G7" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C8" s="15">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
       <c r="D8" s="15">
         <v>8.47</v>
@@ -2279,15 +2270,15 @@
         <f>C8*D8</f>
       </c>
       <c r="G8" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C9" s="15">
         <v>2.3</v>
@@ -2302,15 +2293,15 @@
         <f>C9*D9</f>
       </c>
       <c r="G9" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C10" s="15">
         <v>2.35</v>
@@ -2325,43 +2316,20 @@
         <f>C10*D10</f>
       </c>
       <c r="G10" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C11" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="D11" s="15">
-        <v>8.47</v>
-      </c>
-      <c r="E11" s="15">
-        <v>0.3</v>
-      </c>
-      <c r="F11" s="16">
-        <f>C11*D11</f>
-      </c>
-      <c r="G11" s="4" t="s">
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="17" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="F12" s="18">
-        <f>SUM(F5:F11)</f>
+      <c r="F11" s="18">
+        <f>SUM(F5:F10)</f>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B14" s="19"/>
       <c r="C14" s="19"/>
@@ -2400,37 +2368,37 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>109</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C5" s="15">
         <v>50.8</v>
@@ -2444,10 +2412,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C6" s="15">
         <v>15.9</v>
@@ -2461,10 +2429,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C7" s="15">
         <v>19.46</v>
@@ -2478,10 +2446,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C8" s="15">
         <v>58.98</v>
@@ -2495,10 +2463,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C9" s="15">
         <v>30.4</v>
@@ -2512,10 +2480,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C10" s="15">
         <v>47.2</v>
@@ -2529,10 +2497,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C11" s="15">
         <v>15.9</v>
@@ -2546,10 +2514,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C12" s="15">
         <v>13.98</v>
@@ -2563,10 +2531,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C13" s="15">
         <v>42.39</v>
@@ -2580,10 +2548,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C14" s="15">
         <v>21.85</v>
@@ -2597,10 +2565,10 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C15" s="15">
         <v>47.4</v>
@@ -2614,10 +2582,10 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C16" s="15">
         <v>15.9</v>
@@ -2631,10 +2599,10 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C17" s="15">
         <v>14.28</v>
@@ -2648,10 +2616,10 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C18" s="15">
         <v>43.3</v>
@@ -2665,10 +2633,10 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C19" s="15">
         <v>22.32</v>
@@ -2682,13 +2650,13 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C20" s="15">
-        <v>40.28</v>
+        <v>41.48</v>
       </c>
       <c r="D20" s="16">
         <v>22.96</v>
@@ -2699,13 +2667,13 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C21" s="15">
-        <v>6.4</v>
+        <v>7.6</v>
       </c>
       <c r="D21" s="16">
         <v>26.86</v>
@@ -2716,16 +2684,16 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C22" s="15">
-        <v>15.9</v>
+        <v>-16.94</v>
       </c>
       <c r="D22" s="16">
-        <v>16.2</v>
+        <v>22.96</v>
       </c>
       <c r="E22" s="20">
         <f>C22*D22</f>
@@ -2733,16 +2701,16 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C23" s="15">
-        <v>17.34</v>
+        <v>16.94</v>
       </c>
       <c r="D23" s="16">
-        <v>16.7</v>
+        <v>26.86</v>
       </c>
       <c r="E23" s="20">
         <f>C23*D23</f>
@@ -2750,16 +2718,16 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C24" s="15">
-        <v>52.57</v>
+        <v>15.9</v>
       </c>
       <c r="D24" s="16">
-        <v>4.42</v>
+        <v>16.2</v>
       </c>
       <c r="E24" s="20">
         <f>C24*D24</f>
@@ -2767,16 +2735,16 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C25" s="15">
-        <v>27.1</v>
+        <v>20.6</v>
       </c>
       <c r="D25" s="16">
-        <v>2.34</v>
+        <v>16.7</v>
       </c>
       <c r="E25" s="20">
         <f>C25*D25</f>
@@ -2784,16 +2752,16 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C26" s="15">
-        <v>38.48</v>
+        <v>62.45</v>
       </c>
       <c r="D26" s="16">
-        <v>22.96</v>
+        <v>4.42</v>
       </c>
       <c r="E26" s="20">
         <f>C26*D26</f>
@@ -2801,16 +2769,16 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C27" s="15">
-        <v>4.6</v>
+        <v>32.19</v>
       </c>
       <c r="D27" s="16">
-        <v>26.86</v>
+        <v>2.34</v>
       </c>
       <c r="E27" s="20">
         <f>C27*D27</f>
@@ -2818,16 +2786,16 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C28" s="15">
-        <v>15.9</v>
+        <v>38.48</v>
       </c>
       <c r="D28" s="16">
-        <v>16.2</v>
+        <v>22.96</v>
       </c>
       <c r="E28" s="20">
         <f>C28*D28</f>
@@ -2835,16 +2803,16 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C29" s="15">
-        <v>12.47</v>
+        <v>4.6</v>
       </c>
       <c r="D29" s="16">
-        <v>16.7</v>
+        <v>26.86</v>
       </c>
       <c r="E29" s="20">
         <f>C29*D29</f>
@@ -2852,16 +2820,16 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C30" s="15">
-        <v>37.79</v>
+        <v>15.9</v>
       </c>
       <c r="D30" s="16">
-        <v>4.42</v>
+        <v>16.2</v>
       </c>
       <c r="E30" s="20">
         <f>C30*D30</f>
@@ -2869,16 +2837,16 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C31" s="15">
-        <v>19.48</v>
+        <v>12.47</v>
       </c>
       <c r="D31" s="16">
-        <v>2.34</v>
+        <v>16.7</v>
       </c>
       <c r="E31" s="20">
         <f>C31*D31</f>
@@ -2886,16 +2854,16 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C32" s="15">
-        <v>45.1</v>
+        <v>37.79</v>
       </c>
       <c r="D32" s="16">
-        <v>22.96</v>
+        <v>4.42</v>
       </c>
       <c r="E32" s="20">
         <f>C32*D32</f>
@@ -2903,16 +2871,16 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C33" s="15">
-        <v>4.7</v>
+        <v>19.48</v>
       </c>
       <c r="D33" s="16">
-        <v>26.86</v>
+        <v>2.34</v>
       </c>
       <c r="E33" s="20">
         <f>C33*D33</f>
@@ -2920,16 +2888,16 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C34" s="15">
-        <v>21.2</v>
+        <v>45.1</v>
       </c>
       <c r="D34" s="16">
-        <v>16.2</v>
+        <v>22.96</v>
       </c>
       <c r="E34" s="20">
         <f>C34*D34</f>
@@ -2937,16 +2905,16 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C35" s="15">
-        <v>15.19</v>
+        <v>4.7</v>
       </c>
       <c r="D35" s="16">
-        <v>16.7</v>
+        <v>26.86</v>
       </c>
       <c r="E35" s="20">
         <f>C35*D35</f>
@@ -2954,16 +2922,16 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C36" s="15">
-        <v>46.04</v>
+        <v>21.2</v>
       </c>
       <c r="D36" s="16">
-        <v>4.42</v>
+        <v>16.2</v>
       </c>
       <c r="E36" s="20">
         <f>C36*D36</f>
@@ -2971,16 +2939,16 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C37" s="15">
-        <v>23.73</v>
+        <v>15.19</v>
       </c>
       <c r="D37" s="16">
-        <v>2.34</v>
+        <v>16.7</v>
       </c>
       <c r="E37" s="20">
         <f>C37*D37</f>
@@ -2988,16 +2956,16 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C38" s="15">
-        <v>16.94</v>
+        <v>46.04</v>
       </c>
       <c r="D38" s="16">
-        <v>26.86</v>
+        <v>4.42</v>
       </c>
       <c r="E38" s="20">
         <f>C38*D38</f>
@@ -3005,16 +2973,16 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C39" s="15">
-        <v>8.4</v>
+        <v>23.73</v>
       </c>
       <c r="D39" s="16">
-        <v>16.2</v>
+        <v>2.34</v>
       </c>
       <c r="E39" s="20">
         <f>C39*D39</f>
@@ -3022,10 +2990,10 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C40" s="15">
         <v>1</v>
@@ -3039,13 +3007,13 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C41" s="15">
-        <v>144.88</v>
+        <v>149.97</v>
       </c>
       <c r="D41" s="16">
         <v>5.59</v>
@@ -3056,7 +3024,7 @@
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B42" s="17" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E42" s="21">
         <f>SUM(E5:E41)</f>
@@ -3064,7 +3032,7 @@
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B43" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E43" s="22">
         <f>E42/148.3</f>
@@ -3072,7 +3040,7 @@
     </row>
     <row r="44" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B44" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -3103,40 +3071,40 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>131</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C5" s="16">
         <f>Acero!$E$42</f>
@@ -3153,10 +3121,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C6" s="15">
         <v>166.17</v>
@@ -3168,15 +3136,15 @@
         <f>C6*D6</f>
       </c>
       <c r="F6" s="4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C7" s="15">
         <v>68.3</v>
@@ -3188,15 +3156,15 @@
         <f>C7*D7</f>
       </c>
       <c r="F7" s="4" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C8" s="15">
         <v>10.77</v>
@@ -3208,15 +3176,15 @@
         <f>C8*D8</f>
       </c>
       <c r="F8" s="4" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C9" s="15">
         <v>234.48</v>
@@ -3228,15 +3196,15 @@
         <f>C9*D9</f>
       </c>
       <c r="F9" s="4" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C10" s="15">
         <v>166.17</v>
@@ -3253,10 +3221,10 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C11" s="15">
         <v>176.94</v>
@@ -3268,18 +3236,18 @@
         <f>C11*D11</f>
       </c>
       <c r="F11" s="4" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C12" s="15">
-        <v>84.37</v>
+        <v>84.38</v>
       </c>
       <c r="D12" s="23">
         <f>(Supuestos!$B$11*(1+Supuestos!$B$5)*(1+Supuestos!$B$9)+Supuestos!$B$8*Supuestos!$B$7)</f>
@@ -3293,13 +3261,13 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C13" s="15">
-        <v>75.39</v>
+        <v>75.4</v>
       </c>
       <c r="D13" s="23">
         <f>Supuestos!$B$16</f>
@@ -3308,15 +3276,15 @@
         <f>C13*D13</f>
       </c>
       <c r="F13" s="4" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C14" s="15">
         <v>8.98</v>
@@ -3328,15 +3296,15 @@
         <f>C14*D14</f>
       </c>
       <c r="F14" s="4" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C15" s="15">
         <v>74.58</v>
@@ -3348,18 +3316,18 @@
         <f>C15*D15</f>
       </c>
       <c r="F15" s="4" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C16" s="15">
-        <v>75.39</v>
+        <v>75.4</v>
       </c>
       <c r="D16" s="23">
         <f>(Supuestos!$B$11*(1+Supuestos!$B$5)*(1+Supuestos!$B$9)+Supuestos!$B$8*Supuestos!$B$7)</f>
@@ -3368,15 +3336,15 @@
         <f>C16*D16</f>
       </c>
       <c r="F16" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C17" s="15">
         <v>73.04</v>
@@ -3388,15 +3356,15 @@
         <f>C17*D17</f>
       </c>
       <c r="F17" s="4" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C18" s="15">
         <v>1</v>
@@ -3408,12 +3376,12 @@
         <f>C18*D18</f>
       </c>
       <c r="F18" s="4" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E19" s="24">
         <f>SUM(E5:E18)</f>
@@ -3445,31 +3413,31 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C5" s="25">
         <v>572.86</v>
@@ -3477,10 +3445,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C6" s="25">
         <v>849.18</v>
@@ -3488,10 +3456,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C7" s="25">
         <v>9471.83</v>
@@ -3499,10 +3467,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="C8" s="25">
         <v>10163.61</v>
@@ -3510,10 +3478,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C9" s="25">
         <v>3924.09</v>
@@ -3521,10 +3489,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C10" s="25">
         <v>12377.21</v>
@@ -3532,10 +3500,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C11" s="25">
         <v>3748.1</v>
@@ -3543,10 +3511,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C12" s="25">
         <v>13180.5</v>
@@ -3554,10 +3522,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C13" s="25">
         <v>5829.69</v>
@@ -3565,10 +3533,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C14" s="25">
         <v>18715.51</v>
@@ -3576,10 +3544,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C15" s="25">
         <v>532.8</v>
@@ -3587,7 +3555,7 @@
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B16" s="17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C16" s="24">
         <f>SUM(C5:C15)</f>
@@ -3623,431 +3591,431 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>192</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D5" s="5">
         <v>8376</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="F5" s="13">
         <v>2000</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D6" s="5">
         <v>595</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="F6" s="13">
         <v>400</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="D7" s="5">
         <v>4483</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="F7" s="13">
         <v>750</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="D8" s="5">
         <v>3910</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="F8" s="13">
         <v>1000</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D9" s="5">
         <v>3447</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="F9" s="13">
         <v>1180</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="D10" s="5">
         <v>992</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="F10" s="13">
         <v>992</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="D11" s="5">
         <v>1504</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="F11" s="13">
         <v>1400</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D12" s="5">
         <v>2061</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="F12" s="13">
         <v>1200</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D13" s="5">
         <v>1242</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="F13" s="13">
         <v>890</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D14" s="5">
         <v>1171</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="F14" s="13">
         <v>320</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="D15" s="5">
         <v>730</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="F15" s="13">
         <v>280</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D16" s="5">
         <v>3245</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="F16" s="13">
         <v>715</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D17" s="5">
         <v>3918</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="F17" s="13">
         <v>700</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="D18" s="5">
         <v>3748</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="F18" s="13">
         <v>850</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D19" s="5">
         <v>8012</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="F19" s="13">
         <v>650</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D20" s="5">
         <v>1681</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="F20" s="13">
         <v>520</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D21" s="5">
         <v>1408</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="F21" s="13">
         <v>340</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="22" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E22" s="4" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="F22" s="5">
         <f>SUMIF(G5:G21,"S",F5:F21)</f>
@@ -4055,7 +4023,7 @@
     </row>
     <row r="23" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E23" s="4" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="F23" s="5">
         <f>SUMIF(G5:G21,"M",F5:F21)</f>
@@ -4063,7 +4031,7 @@
     </row>
     <row r="24" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E24" s="4" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="F24" s="5">
         <f>SUMIF(G5:G21,"A",F5:F21)</f>
@@ -4071,7 +4039,7 @@
     </row>
     <row r="25" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E25" s="17" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="F25" s="24">
         <f>SUM(F5:F21)</f>
@@ -4079,7 +4047,7 @@
     </row>
     <row r="26" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E26" s="17" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="F26" s="24">
         <f>F25*(1+Supuestos!$B$31)</f>
@@ -4087,7 +4055,7 @@
     </row>
     <row r="27" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E27" s="17" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="F27" s="24">
         <f>'Resumen piloto'!B15-F26</f>
@@ -4119,17 +4087,17 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>28</v>
@@ -4140,29 +4108,29 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="B5" s="14">
         <v>6</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="B6" s="12">
         <v>146.7</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="B7" s="13">
         <v>28250</v>
@@ -4173,139 +4141,139 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="B8" s="10">
         <v>0.08</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="B9" s="13">
         <v>8000</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="B10" s="10">
         <v>0.01</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="B11" s="10">
         <v>0.03</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B12" s="13">
         <v>190091</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B13" s="13">
         <v>194636</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="B14" s="13">
         <v>225400</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="B15" s="13">
         <v>273600</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="B16" s="13">
         <v>209100</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="B17" s="13">
         <v>214100</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="B19" s="20">
-        <f>(Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.59*Supuestos!$B$8*Supuestos!$B$7)/Supuestos!$B$7</f>
+        <f>(Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.61*Supuestos!$B$8*Supuestos!$B$7)/Supuestos!$B$7</f>
       </c>
       <c r="F19" s="4" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="B20" s="16">
         <f>$B$5*$B$6/$B$19</f>
       </c>
       <c r="F20" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="B21" s="22">
         <f>16/$B$20</f>
@@ -4316,18 +4284,18 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="B22" s="5">
         <f>$B$7*$B$5/9</f>
       </c>
       <c r="F22" s="4" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -4335,44 +4303,44 @@
         <v>2</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B26" s="5">
-        <f>((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.59*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8</f>
+        <f>((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.61*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8</f>
       </c>
       <c r="C26" s="5">
-        <f>((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.59*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8</f>
+        <f>((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.61*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8</f>
       </c>
       <c r="D26" s="5">
-        <f>((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.59*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8</f>
+        <f>((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.61*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8</f>
       </c>
       <c r="E26" s="5">
-        <f>((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.59*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8</f>
+        <f>((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.61*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8</f>
       </c>
       <c r="F26" s="4" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="B27" s="5">
         <f>Supuestos!$B$28*Supuestos!$B$5/Supuestos!$B$29</f>
@@ -4387,12 +4355,12 @@
         <f>Supuestos!$B$28*Supuestos!$B$5/Supuestos!$B$29</f>
       </c>
       <c r="F27" s="4" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B28" s="5">
         <f>Supuestos!$B$28*(1+Supuestos!$B$5)*(1/$B$20-1/Supuestos!$B$29)</f>
@@ -4407,18 +4375,18 @@
         <f>Supuestos!$B$28*(1+Supuestos!$B$5)*(1/$B$20-1/Supuestos!$B$29)</f>
       </c>
       <c r="F28" s="4" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B29" s="5">
         <f>0</f>
       </c>
       <c r="C29" s="5">
-        <f>MAX(0,$B$22*(1+$B$8)*Supuestos!$B$30-((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.59*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*(1+$B$8))</f>
+        <f>MAX(0,$B$22*(1+$B$8)*Supuestos!$B$30-((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.61*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*(1+$B$8))</f>
       </c>
       <c r="D29" s="5">
         <f>0</f>
@@ -4427,12 +4395,12 @@
         <f>0</f>
       </c>
       <c r="F29" s="4" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="B30" s="5">
         <f>$B$9/$B$20</f>
@@ -4447,12 +4415,12 @@
         <f>$B$9/$B$20</f>
       </c>
       <c r="F30" s="4" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="B31" s="5">
         <f>('Resumen piloto'!$B$13+SUM(B26:B30))*$B$10</f>
@@ -4469,7 +4437,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="B32" s="5">
         <f>('Resumen piloto'!$B$13+SUM(B26:B30))*$B$11</f>
@@ -4486,7 +4454,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="17" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="B33" s="5">
         <f>SUM(B26:B32)</f>
@@ -4503,7 +4471,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="B34" s="5">
         <f>'Resumen piloto'!$B$13</f>
@@ -4520,7 +4488,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="B35" s="7">
         <f>B33+B34</f>
@@ -4537,7 +4505,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="B36" s="5">
         <f>$B$14</f>
@@ -4554,7 +4522,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="B37" s="26">
         <f>1-B34/B36</f>
@@ -4571,7 +4539,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="B38" s="7">
         <f>B36-B35</f>
@@ -4588,7 +4556,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="17" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="B39" s="27">
         <f>B38/B36</f>
@@ -4605,32 +4573,32 @@
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="17" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="F42" s="3" t="s">
         <v>320</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>296</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="D42" s="3" t="s">
-        <v>321</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="B43" s="5">
         <f>B35*(1+0)</f>
@@ -4650,7 +4618,7 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="B44" s="5">
         <f>B35*(1+0.05)</f>
@@ -4670,7 +4638,7 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="B45" s="5">
         <f>B35*(1+0.08)</f>
@@ -4690,7 +4658,7 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="B46" s="5">
         <f>B35*(1+0.1)</f>
@@ -4710,7 +4678,7 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="B47" s="5">
         <f>B35*(1+0.12)</f>
@@ -4730,7 +4698,7 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B48" s="5">
         <f>B35*(1+0.15)</f>
@@ -4750,7 +4718,7 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="B49" s="5">
         <f>B35*(1+0.21951219512195122)</f>
@@ -4770,7 +4738,7 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="B50" s="5">
         <f>B35*(1+0.25)</f>
@@ -4790,27 +4758,27 @@
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="17" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="53" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="D53" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="B53" s="3" t="s">
+      <c r="E53" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="C53" s="3" t="s">
+      <c r="F53" s="3" t="s">
         <v>335</v>
-      </c>
-      <c r="D53" s="3" t="s">
-        <v>336</v>
-      </c>
-      <c r="E53" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="F53" s="3" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -4824,7 +4792,7 @@
         <f>16/(6*$B$6/$B$19)</f>
       </c>
       <c r="D54" s="5">
-        <f>($B$12-Supuestos!$B$28/Supuestos!$B$29+((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.59*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8+(Supuestos!$B$28*(1+Supuestos!$B$5)+$B$9)/(6*$B$6/$B$19))*(1+$B$10+$B$11)</f>
+        <f>($B$12-Supuestos!$B$28/Supuestos!$B$29+((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.61*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8+(Supuestos!$B$28*(1+Supuestos!$B$5)+$B$9)/(6*$B$6/$B$19))*(1+$B$10+$B$11)</f>
       </c>
       <c r="E54" s="5">
         <f>$B$16-D54</f>
@@ -4844,7 +4812,7 @@
         <f>16/(9*$B$6/$B$19)</f>
       </c>
       <c r="D55" s="5">
-        <f>($B$12-Supuestos!$B$28/Supuestos!$B$29+((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.59*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8+(Supuestos!$B$28*(1+Supuestos!$B$5)+$B$9)/(9*$B$6/$B$19))*(1+$B$10+$B$11)</f>
+        <f>($B$12-Supuestos!$B$28/Supuestos!$B$29+((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.61*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8+(Supuestos!$B$28*(1+Supuestos!$B$5)+$B$9)/(9*$B$6/$B$19))*(1+$B$10+$B$11)</f>
       </c>
       <c r="E55" s="5">
         <f>$B$16-D55</f>
@@ -4864,7 +4832,7 @@
         <f>16/(12*$B$6/$B$19)</f>
       </c>
       <c r="D56" s="5">
-        <f>($B$12-Supuestos!$B$28/Supuestos!$B$29+((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.59*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8+(Supuestos!$B$28*(1+Supuestos!$B$5)+$B$9)/(12*$B$6/$B$19))*(1+$B$10+$B$11)</f>
+        <f>($B$12-Supuestos!$B$28/Supuestos!$B$29+((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.61*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8+(Supuestos!$B$28*(1+Supuestos!$B$5)+$B$9)/(12*$B$6/$B$19))*(1+$B$10+$B$11)</f>
       </c>
       <c r="E56" s="5">
         <f>$B$16-D56</f>
@@ -4884,7 +4852,7 @@
         <f>16/(15*$B$6/$B$19)</f>
       </c>
       <c r="D57" s="5">
-        <f>($B$12-Supuestos!$B$28/Supuestos!$B$29+((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.59*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8+(Supuestos!$B$28*(1+Supuestos!$B$5)+$B$9)/(15*$B$6/$B$19))*(1+$B$10+$B$11)</f>
+        <f>($B$12-Supuestos!$B$28/Supuestos!$B$29+((Acero!$E$42*(Supuestos!$B$6-0.90-0.24)+479.61*Supuestos!$B$8*Supuestos!$B$7)+Supuestos!$B$25*Supuestos!$B$7*(1+Supuestos!$B$26))*$B$8+(Supuestos!$B$28*(1+Supuestos!$B$5)+$B$9)/(15*$B$6/$B$19))*(1+$B$10+$B$11)</f>
       </c>
       <c r="E57" s="5">
         <f>$B$16-D57</f>
@@ -4905,7 +4873,7 @@
     </row>
     <row r="60" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="B60" s="9"/>
       <c r="C60" s="9"/>
@@ -4915,7 +4883,7 @@
     </row>
     <row r="61" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="9" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="B61" s="9"/>
       <c r="C61" s="9"/>
@@ -4925,7 +4893,7 @@
     </row>
     <row r="62" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="9" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="B62" s="9"/>
       <c r="C62" s="9"/>
@@ -4935,7 +4903,7 @@
     </row>
     <row r="63" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="9" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="B63" s="9"/>
       <c r="C63" s="9"/>
@@ -4945,7 +4913,7 @@
     </row>
     <row r="64" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="9" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="B64" s="9"/>
       <c r="C64" s="9"/>
@@ -4955,7 +4923,7 @@
     </row>
     <row r="65" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="9" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>

</xml_diff>